<commit_message>
Upset higher seeds: record vs top 40 counts November games only
</commit_message>
<xml_diff>
--- a/reports/upset_high_seeds.xlsx
+++ b/reports/upset_high_seeds.xlsx
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>169 games (First Four not included). November = the team's games in November of that season. Top 40 = that season's pre-tournament top 40 by Strongside net rating; record from games before the tournament.</t>
+          <t>169 games (First Four not included). November = the team's games in November of that season. Top 40 = that season's pre-tournament top 40 by Strongside net rating; the top-40 record counts November games only.</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>No games vs top 40 (not battle tested)</t>
+          <t>No November games vs top 40 (not battle tested)</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -628,22 +628,22 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Top-40 W</t>
+          <t>Nov top-40 W</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Top-40 L</t>
+          <t>Nov top-40 L</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>Record vs top 40</t>
+          <t>November record vs top 40</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>Top-40 games</t>
+          <t>Nov top-40 games</t>
         </is>
       </c>
     </row>
@@ -688,10 +688,10 @@
         <v/>
       </c>
       <c r="K6" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M6" s="8">
         <f>K6&amp;"-"&amp;L6</f>
@@ -743,10 +743,10 @@
         <v/>
       </c>
       <c r="K7" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M7" s="8">
         <f>K7&amp;"-"&amp;L7</f>
@@ -798,10 +798,10 @@
         <v/>
       </c>
       <c r="K8" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="8">
         <f>K8&amp;"-"&amp;L8</f>
@@ -853,10 +853,10 @@
         <v/>
       </c>
       <c r="K9" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M9" s="8">
         <f>K9&amp;"-"&amp;L9</f>
@@ -908,10 +908,10 @@
         <v/>
       </c>
       <c r="K10" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="M10" s="8">
         <f>K10&amp;"-"&amp;L10</f>
@@ -963,10 +963,10 @@
         <v/>
       </c>
       <c r="K11" s="8" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" s="8">
         <f>K11&amp;"-"&amp;L11</f>
@@ -1018,10 +1018,10 @@
         <v/>
       </c>
       <c r="K12" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M12" s="8">
         <f>K12&amp;"-"&amp;L12</f>
@@ -1073,7 +1073,7 @@
         <v/>
       </c>
       <c r="K13" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>0</v>
@@ -1128,10 +1128,10 @@
         <v/>
       </c>
       <c r="K14" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M14" s="8">
         <f>K14&amp;"-"&amp;L14</f>
@@ -1183,10 +1183,10 @@
         <v/>
       </c>
       <c r="K15" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L15" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M15" s="8">
         <f>K15&amp;"-"&amp;L15</f>
@@ -1238,10 +1238,10 @@
         <v/>
       </c>
       <c r="K16" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M16" s="8">
         <f>K16&amp;"-"&amp;L16</f>
@@ -1293,10 +1293,10 @@
         <v/>
       </c>
       <c r="K17" s="8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M17" s="8">
         <f>K17&amp;"-"&amp;L17</f>
@@ -1348,10 +1348,10 @@
         <v/>
       </c>
       <c r="K18" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L18" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M18" s="8">
         <f>K18&amp;"-"&amp;L18</f>
@@ -1403,10 +1403,10 @@
         <v/>
       </c>
       <c r="K19" s="8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M19" s="8">
         <f>K19&amp;"-"&amp;L19</f>
@@ -1458,10 +1458,10 @@
         <v/>
       </c>
       <c r="K20" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M20" s="8">
         <f>K20&amp;"-"&amp;L20</f>
@@ -1513,10 +1513,10 @@
         <v/>
       </c>
       <c r="K21" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L21" s="8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M21" s="8">
         <f>K21&amp;"-"&amp;L21</f>
@@ -1568,10 +1568,10 @@
         <v/>
       </c>
       <c r="K22" s="8" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M22" s="8">
         <f>K22&amp;"-"&amp;L22</f>
@@ -1623,10 +1623,10 @@
         <v/>
       </c>
       <c r="K23" s="8" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M23" s="8">
         <f>K23&amp;"-"&amp;L23</f>
@@ -1678,10 +1678,10 @@
         <v/>
       </c>
       <c r="K24" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M24" s="8">
         <f>K24&amp;"-"&amp;L24</f>
@@ -1733,10 +1733,10 @@
         <v/>
       </c>
       <c r="K25" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L25" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M25" s="8">
         <f>K25&amp;"-"&amp;L25</f>
@@ -1788,10 +1788,10 @@
         <v/>
       </c>
       <c r="K26" s="8" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="L26" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M26" s="8">
         <f>K26&amp;"-"&amp;L26</f>
@@ -1843,10 +1843,10 @@
         <v/>
       </c>
       <c r="K27" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L27" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M27" s="8">
         <f>K27&amp;"-"&amp;L27</f>
@@ -1898,10 +1898,10 @@
         <v/>
       </c>
       <c r="K28" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L28" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M28" s="8">
         <f>K28&amp;"-"&amp;L28</f>
@@ -1953,10 +1953,10 @@
         <v/>
       </c>
       <c r="K29" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L29" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M29" s="8">
         <f>K29&amp;"-"&amp;L29</f>
@@ -2008,10 +2008,10 @@
         <v/>
       </c>
       <c r="K30" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L30" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M30" s="8">
         <f>K30&amp;"-"&amp;L30</f>
@@ -2063,10 +2063,10 @@
         <v/>
       </c>
       <c r="K31" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L31" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M31" s="8">
         <f>K31&amp;"-"&amp;L31</f>
@@ -2118,10 +2118,10 @@
         <v/>
       </c>
       <c r="K32" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L32" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M32" s="8">
         <f>K32&amp;"-"&amp;L32</f>
@@ -2173,10 +2173,10 @@
         <v/>
       </c>
       <c r="K33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="8" t="n">
         <v>2</v>
-      </c>
-      <c r="L33" s="8" t="n">
-        <v>3</v>
       </c>
       <c r="M33" s="8">
         <f>K33&amp;"-"&amp;L33</f>
@@ -2228,10 +2228,10 @@
         <v/>
       </c>
       <c r="K34" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L34" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M34" s="8">
         <f>K34&amp;"-"&amp;L34</f>
@@ -2283,10 +2283,10 @@
         <v/>
       </c>
       <c r="K35" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L35" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M35" s="8">
         <f>K35&amp;"-"&amp;L35</f>
@@ -2338,10 +2338,10 @@
         <v/>
       </c>
       <c r="K36" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L36" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M36" s="8">
         <f>K36&amp;"-"&amp;L36</f>
@@ -2393,10 +2393,10 @@
         <v/>
       </c>
       <c r="K37" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L37" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M37" s="8">
         <f>K37&amp;"-"&amp;L37</f>
@@ -2448,10 +2448,10 @@
         <v/>
       </c>
       <c r="K38" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L38" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M38" s="8">
         <f>K38&amp;"-"&amp;L38</f>
@@ -2503,10 +2503,10 @@
         <v/>
       </c>
       <c r="K39" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L39" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M39" s="8">
         <f>K39&amp;"-"&amp;L39</f>
@@ -2558,10 +2558,10 @@
         <v/>
       </c>
       <c r="K40" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L40" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M40" s="8">
         <f>K40&amp;"-"&amp;L40</f>
@@ -2613,10 +2613,10 @@
         <v/>
       </c>
       <c r="K41" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L41" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M41" s="8">
         <f>K41&amp;"-"&amp;L41</f>
@@ -2668,10 +2668,10 @@
         <v/>
       </c>
       <c r="K42" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L42" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M42" s="8">
         <f>K42&amp;"-"&amp;L42</f>
@@ -2723,10 +2723,10 @@
         <v/>
       </c>
       <c r="K43" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L43" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M43" s="8">
         <f>K43&amp;"-"&amp;L43</f>
@@ -2778,10 +2778,10 @@
         <v/>
       </c>
       <c r="K44" s="8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L44" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="M44" s="8">
         <f>K44&amp;"-"&amp;L44</f>
@@ -2833,10 +2833,10 @@
         <v/>
       </c>
       <c r="K45" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L45" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M45" s="8">
         <f>K45&amp;"-"&amp;L45</f>
@@ -2888,10 +2888,10 @@
         <v/>
       </c>
       <c r="K46" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L46" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M46" s="8">
         <f>K46&amp;"-"&amp;L46</f>
@@ -2943,7 +2943,7 @@
         <v/>
       </c>
       <c r="K47" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L47" s="8" t="n">
         <v>1</v>
@@ -2998,10 +2998,10 @@
         <v/>
       </c>
       <c r="K48" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L48" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M48" s="8">
         <f>K48&amp;"-"&amp;L48</f>
@@ -3053,10 +3053,10 @@
         <v/>
       </c>
       <c r="K49" s="8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L49" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M49" s="8">
         <f>K49&amp;"-"&amp;L49</f>
@@ -3108,10 +3108,10 @@
         <v/>
       </c>
       <c r="K50" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L50" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M50" s="8">
         <f>K50&amp;"-"&amp;L50</f>
@@ -3163,10 +3163,10 @@
         <v/>
       </c>
       <c r="K51" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L51" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M51" s="8">
         <f>K51&amp;"-"&amp;L51</f>
@@ -3218,10 +3218,10 @@
         <v/>
       </c>
       <c r="K52" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L52" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M52" s="8">
         <f>K52&amp;"-"&amp;L52</f>
@@ -3273,10 +3273,10 @@
         <v/>
       </c>
       <c r="K53" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L53" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M53" s="8">
         <f>K53&amp;"-"&amp;L53</f>
@@ -3328,10 +3328,10 @@
         <v/>
       </c>
       <c r="K54" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L54" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M54" s="8">
         <f>K54&amp;"-"&amp;L54</f>
@@ -3383,10 +3383,10 @@
         <v/>
       </c>
       <c r="K55" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L55" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M55" s="8">
         <f>K55&amp;"-"&amp;L55</f>
@@ -3438,7 +3438,7 @@
         <v/>
       </c>
       <c r="K56" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L56" s="8" t="n">
         <v>0</v>
@@ -3493,10 +3493,10 @@
         <v/>
       </c>
       <c r="K57" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L57" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M57" s="8">
         <f>K57&amp;"-"&amp;L57</f>
@@ -3548,10 +3548,10 @@
         <v/>
       </c>
       <c r="K58" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L58" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M58" s="8">
         <f>K58&amp;"-"&amp;L58</f>
@@ -3603,10 +3603,10 @@
         <v/>
       </c>
       <c r="K59" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L59" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M59" s="8">
         <f>K59&amp;"-"&amp;L59</f>
@@ -3658,10 +3658,10 @@
         <v/>
       </c>
       <c r="K60" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L60" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M60" s="8">
         <f>K60&amp;"-"&amp;L60</f>
@@ -3713,10 +3713,10 @@
         <v/>
       </c>
       <c r="K61" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L61" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M61" s="8">
         <f>K61&amp;"-"&amp;L61</f>
@@ -3768,10 +3768,10 @@
         <v/>
       </c>
       <c r="K62" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L62" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M62" s="8">
         <f>K62&amp;"-"&amp;L62</f>
@@ -3823,10 +3823,10 @@
         <v/>
       </c>
       <c r="K63" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L63" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M63" s="8">
         <f>K63&amp;"-"&amp;L63</f>
@@ -3878,10 +3878,10 @@
         <v/>
       </c>
       <c r="K64" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L64" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M64" s="8">
         <f>K64&amp;"-"&amp;L64</f>
@@ -3933,10 +3933,10 @@
         <v/>
       </c>
       <c r="K65" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L65" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M65" s="8">
         <f>K65&amp;"-"&amp;L65</f>
@@ -3988,10 +3988,10 @@
         <v/>
       </c>
       <c r="K66" s="8" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L66" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M66" s="8">
         <f>K66&amp;"-"&amp;L66</f>
@@ -4098,10 +4098,10 @@
         <v/>
       </c>
       <c r="K68" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L68" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M68" s="8">
         <f>K68&amp;"-"&amp;L68</f>
@@ -4153,10 +4153,10 @@
         <v/>
       </c>
       <c r="K69" s="8" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L69" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M69" s="8">
         <f>K69&amp;"-"&amp;L69</f>
@@ -4208,10 +4208,10 @@
         <v/>
       </c>
       <c r="K70" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L70" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M70" s="8">
         <f>K70&amp;"-"&amp;L70</f>
@@ -4263,10 +4263,10 @@
         <v/>
       </c>
       <c r="K71" s="8" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="L71" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M71" s="8">
         <f>K71&amp;"-"&amp;L71</f>
@@ -4318,10 +4318,10 @@
         <v/>
       </c>
       <c r="K72" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L72" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M72" s="8">
         <f>K72&amp;"-"&amp;L72</f>
@@ -4373,10 +4373,10 @@
         <v/>
       </c>
       <c r="K73" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L73" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M73" s="8">
         <f>K73&amp;"-"&amp;L73</f>
@@ -4428,10 +4428,10 @@
         <v/>
       </c>
       <c r="K74" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L74" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M74" s="8">
         <f>K74&amp;"-"&amp;L74</f>
@@ -4483,10 +4483,10 @@
         <v/>
       </c>
       <c r="K75" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L75" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M75" s="8">
         <f>K75&amp;"-"&amp;L75</f>
@@ -4538,10 +4538,10 @@
         <v/>
       </c>
       <c r="K76" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L76" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M76" s="8">
         <f>K76&amp;"-"&amp;L76</f>
@@ -4593,10 +4593,10 @@
         <v/>
       </c>
       <c r="K77" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L77" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M77" s="8">
         <f>K77&amp;"-"&amp;L77</f>
@@ -4648,10 +4648,10 @@
         <v/>
       </c>
       <c r="K78" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L78" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M78" s="8">
         <f>K78&amp;"-"&amp;L78</f>
@@ -4703,10 +4703,10 @@
         <v/>
       </c>
       <c r="K79" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L79" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M79" s="8">
         <f>K79&amp;"-"&amp;L79</f>
@@ -4758,10 +4758,10 @@
         <v/>
       </c>
       <c r="K80" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L80" s="8" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="M80" s="8">
         <f>K80&amp;"-"&amp;L80</f>
@@ -4813,10 +4813,10 @@
         <v/>
       </c>
       <c r="K81" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L81" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M81" s="8">
         <f>K81&amp;"-"&amp;L81</f>
@@ -4868,10 +4868,10 @@
         <v/>
       </c>
       <c r="K82" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L82" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M82" s="8">
         <f>K82&amp;"-"&amp;L82</f>
@@ -4923,10 +4923,10 @@
         <v/>
       </c>
       <c r="K83" s="8" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L83" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M83" s="8">
         <f>K83&amp;"-"&amp;L83</f>
@@ -4978,10 +4978,10 @@
         <v/>
       </c>
       <c r="K84" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L84" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M84" s="8">
         <f>K84&amp;"-"&amp;L84</f>
@@ -5033,10 +5033,10 @@
         <v/>
       </c>
       <c r="K85" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L85" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M85" s="8">
         <f>K85&amp;"-"&amp;L85</f>
@@ -5088,10 +5088,10 @@
         <v/>
       </c>
       <c r="K86" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L86" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M86" s="8">
         <f>K86&amp;"-"&amp;L86</f>
@@ -5143,10 +5143,10 @@
         <v/>
       </c>
       <c r="K87" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L87" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M87" s="8">
         <f>K87&amp;"-"&amp;L87</f>
@@ -5198,10 +5198,10 @@
         <v/>
       </c>
       <c r="K88" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L88" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M88" s="8">
         <f>K88&amp;"-"&amp;L88</f>
@@ -5253,10 +5253,10 @@
         <v/>
       </c>
       <c r="K89" s="8" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L89" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M89" s="8">
         <f>K89&amp;"-"&amp;L89</f>
@@ -5308,10 +5308,10 @@
         <v/>
       </c>
       <c r="K90" s="8" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L90" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M90" s="8">
         <f>K90&amp;"-"&amp;L90</f>
@@ -5363,10 +5363,10 @@
         <v/>
       </c>
       <c r="K91" s="8" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="L91" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M91" s="8">
         <f>K91&amp;"-"&amp;L91</f>
@@ -5418,10 +5418,10 @@
         <v/>
       </c>
       <c r="K92" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L92" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M92" s="8">
         <f>K92&amp;"-"&amp;L92</f>
@@ -5473,10 +5473,10 @@
         <v/>
       </c>
       <c r="K93" s="8" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L93" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M93" s="8">
         <f>K93&amp;"-"&amp;L93</f>
@@ -5528,10 +5528,10 @@
         <v/>
       </c>
       <c r="K94" s="8" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L94" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M94" s="8">
         <f>K94&amp;"-"&amp;L94</f>
@@ -5583,7 +5583,7 @@
         <v/>
       </c>
       <c r="K95" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L95" s="8" t="n">
         <v>2</v>
@@ -5638,10 +5638,10 @@
         <v/>
       </c>
       <c r="K96" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L96" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M96" s="8">
         <f>K96&amp;"-"&amp;L96</f>
@@ -5693,10 +5693,10 @@
         <v/>
       </c>
       <c r="K97" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L97" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M97" s="8">
         <f>K97&amp;"-"&amp;L97</f>
@@ -5748,10 +5748,10 @@
         <v/>
       </c>
       <c r="K98" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L98" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M98" s="8">
         <f>K98&amp;"-"&amp;L98</f>
@@ -5803,10 +5803,10 @@
         <v/>
       </c>
       <c r="K99" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L99" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M99" s="8">
         <f>K99&amp;"-"&amp;L99</f>
@@ -5858,10 +5858,10 @@
         <v/>
       </c>
       <c r="K100" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L100" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M100" s="8">
         <f>K100&amp;"-"&amp;L100</f>
@@ -5913,10 +5913,10 @@
         <v/>
       </c>
       <c r="K101" s="8" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="L101" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="M101" s="8">
         <f>K101&amp;"-"&amp;L101</f>
@@ -5968,10 +5968,10 @@
         <v/>
       </c>
       <c r="K102" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L102" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M102" s="8">
         <f>K102&amp;"-"&amp;L102</f>
@@ -6023,10 +6023,10 @@
         <v/>
       </c>
       <c r="K103" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L103" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M103" s="8">
         <f>K103&amp;"-"&amp;L103</f>
@@ -6078,10 +6078,10 @@
         <v/>
       </c>
       <c r="K104" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L104" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M104" s="8">
         <f>K104&amp;"-"&amp;L104</f>
@@ -6133,10 +6133,10 @@
         <v/>
       </c>
       <c r="K105" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L105" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M105" s="8">
         <f>K105&amp;"-"&amp;L105</f>
@@ -6191,7 +6191,7 @@
         <v>0</v>
       </c>
       <c r="L106" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M106" s="8">
         <f>K106&amp;"-"&amp;L106</f>
@@ -6243,10 +6243,10 @@
         <v/>
       </c>
       <c r="K107" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L107" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M107" s="8">
         <f>K107&amp;"-"&amp;L107</f>
@@ -6298,10 +6298,10 @@
         <v/>
       </c>
       <c r="K108" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L108" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M108" s="8">
         <f>K108&amp;"-"&amp;L108</f>
@@ -6353,10 +6353,10 @@
         <v/>
       </c>
       <c r="K109" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L109" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M109" s="8">
         <f>K109&amp;"-"&amp;L109</f>
@@ -6408,10 +6408,10 @@
         <v/>
       </c>
       <c r="K110" s="8" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L110" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M110" s="8">
         <f>K110&amp;"-"&amp;L110</f>
@@ -6463,10 +6463,10 @@
         <v/>
       </c>
       <c r="K111" s="8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L111" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M111" s="8">
         <f>K111&amp;"-"&amp;L111</f>
@@ -6518,10 +6518,10 @@
         <v/>
       </c>
       <c r="K112" s="8" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L112" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M112" s="8">
         <f>K112&amp;"-"&amp;L112</f>
@@ -6573,10 +6573,10 @@
         <v/>
       </c>
       <c r="K113" s="8" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L113" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M113" s="8">
         <f>K113&amp;"-"&amp;L113</f>
@@ -6628,10 +6628,10 @@
         <v/>
       </c>
       <c r="K114" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L114" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M114" s="8">
         <f>K114&amp;"-"&amp;L114</f>
@@ -6683,10 +6683,10 @@
         <v/>
       </c>
       <c r="K115" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L115" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M115" s="8">
         <f>K115&amp;"-"&amp;L115</f>
@@ -6738,10 +6738,10 @@
         <v/>
       </c>
       <c r="K116" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L116" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M116" s="8">
         <f>K116&amp;"-"&amp;L116</f>
@@ -6793,10 +6793,10 @@
         <v/>
       </c>
       <c r="K117" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L117" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M117" s="8">
         <f>K117&amp;"-"&amp;L117</f>
@@ -6851,7 +6851,7 @@
         <v>1</v>
       </c>
       <c r="L118" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M118" s="8">
         <f>K118&amp;"-"&amp;L118</f>
@@ -6903,10 +6903,10 @@
         <v/>
       </c>
       <c r="K119" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L119" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M119" s="8">
         <f>K119&amp;"-"&amp;L119</f>
@@ -6958,10 +6958,10 @@
         <v/>
       </c>
       <c r="K120" s="8" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L120" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M120" s="8">
         <f>K120&amp;"-"&amp;L120</f>
@@ -7013,10 +7013,10 @@
         <v/>
       </c>
       <c r="K121" s="8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L121" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M121" s="8">
         <f>K121&amp;"-"&amp;L121</f>
@@ -7068,10 +7068,10 @@
         <v/>
       </c>
       <c r="K122" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L122" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M122" s="8">
         <f>K122&amp;"-"&amp;L122</f>
@@ -7123,10 +7123,10 @@
         <v/>
       </c>
       <c r="K123" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L123" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M123" s="8">
         <f>K123&amp;"-"&amp;L123</f>
@@ -7178,10 +7178,10 @@
         <v/>
       </c>
       <c r="K124" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L124" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M124" s="8">
         <f>K124&amp;"-"&amp;L124</f>
@@ -7233,10 +7233,10 @@
         <v/>
       </c>
       <c r="K125" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L125" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M125" s="8">
         <f>K125&amp;"-"&amp;L125</f>
@@ -7291,7 +7291,7 @@
         <v>0</v>
       </c>
       <c r="L126" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M126" s="8">
         <f>K126&amp;"-"&amp;L126</f>
@@ -7343,10 +7343,10 @@
         <v/>
       </c>
       <c r="K127" s="8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L127" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M127" s="8">
         <f>K127&amp;"-"&amp;L127</f>
@@ -7398,10 +7398,10 @@
         <v/>
       </c>
       <c r="K128" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L128" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M128" s="8">
         <f>K128&amp;"-"&amp;L128</f>
@@ -7453,10 +7453,10 @@
         <v/>
       </c>
       <c r="K129" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L129" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M129" s="8">
         <f>K129&amp;"-"&amp;L129</f>
@@ -7508,10 +7508,10 @@
         <v/>
       </c>
       <c r="K130" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L130" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M130" s="8">
         <f>K130&amp;"-"&amp;L130</f>
@@ -7563,10 +7563,10 @@
         <v/>
       </c>
       <c r="K131" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L131" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M131" s="8">
         <f>K131&amp;"-"&amp;L131</f>
@@ -7618,10 +7618,10 @@
         <v/>
       </c>
       <c r="K132" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L132" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M132" s="8">
         <f>K132&amp;"-"&amp;L132</f>
@@ -7673,10 +7673,10 @@
         <v/>
       </c>
       <c r="K133" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L133" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M133" s="8">
         <f>K133&amp;"-"&amp;L133</f>
@@ -7728,10 +7728,10 @@
         <v/>
       </c>
       <c r="K134" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L134" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M134" s="8">
         <f>K134&amp;"-"&amp;L134</f>
@@ -7783,10 +7783,10 @@
         <v/>
       </c>
       <c r="K135" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L135" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M135" s="8">
         <f>K135&amp;"-"&amp;L135</f>
@@ -7838,10 +7838,10 @@
         <v/>
       </c>
       <c r="K136" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L136" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M136" s="8">
         <f>K136&amp;"-"&amp;L136</f>
@@ -7893,10 +7893,10 @@
         <v/>
       </c>
       <c r="K137" s="8" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L137" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M137" s="8">
         <f>K137&amp;"-"&amp;L137</f>
@@ -7948,10 +7948,10 @@
         <v/>
       </c>
       <c r="K138" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L138" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M138" s="8">
         <f>K138&amp;"-"&amp;L138</f>
@@ -8003,10 +8003,10 @@
         <v/>
       </c>
       <c r="K139" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L139" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M139" s="8">
         <f>K139&amp;"-"&amp;L139</f>
@@ -8058,10 +8058,10 @@
         <v/>
       </c>
       <c r="K140" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L140" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M140" s="8">
         <f>K140&amp;"-"&amp;L140</f>
@@ -8113,10 +8113,10 @@
         <v/>
       </c>
       <c r="K141" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L141" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M141" s="8">
         <f>K141&amp;"-"&amp;L141</f>
@@ -8168,10 +8168,10 @@
         <v/>
       </c>
       <c r="K142" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L142" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M142" s="8">
         <f>K142&amp;"-"&amp;L142</f>
@@ -8223,10 +8223,10 @@
         <v/>
       </c>
       <c r="K143" s="8" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="L143" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M143" s="8">
         <f>K143&amp;"-"&amp;L143</f>
@@ -8278,10 +8278,10 @@
         <v/>
       </c>
       <c r="K144" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L144" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M144" s="8">
         <f>K144&amp;"-"&amp;L144</f>
@@ -8333,10 +8333,10 @@
         <v/>
       </c>
       <c r="K145" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L145" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M145" s="8">
         <f>K145&amp;"-"&amp;L145</f>
@@ -8388,10 +8388,10 @@
         <v/>
       </c>
       <c r="K146" s="8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L146" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M146" s="8">
         <f>K146&amp;"-"&amp;L146</f>
@@ -8443,10 +8443,10 @@
         <v/>
       </c>
       <c r="K147" s="8" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="L147" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M147" s="8">
         <f>K147&amp;"-"&amp;L147</f>
@@ -8498,10 +8498,10 @@
         <v/>
       </c>
       <c r="K148" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L148" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M148" s="8">
         <f>K148&amp;"-"&amp;L148</f>
@@ -8553,10 +8553,10 @@
         <v/>
       </c>
       <c r="K149" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L149" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M149" s="8">
         <f>K149&amp;"-"&amp;L149</f>
@@ -8608,10 +8608,10 @@
         <v/>
       </c>
       <c r="K150" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L150" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M150" s="8">
         <f>K150&amp;"-"&amp;L150</f>
@@ -8663,10 +8663,10 @@
         <v/>
       </c>
       <c r="K151" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="L151" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M151" s="8">
         <f>K151&amp;"-"&amp;L151</f>
@@ -8718,10 +8718,10 @@
         <v/>
       </c>
       <c r="K152" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L152" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M152" s="8">
         <f>K152&amp;"-"&amp;L152</f>
@@ -8773,10 +8773,10 @@
         <v/>
       </c>
       <c r="K153" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L153" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M153" s="8">
         <f>K153&amp;"-"&amp;L153</f>
@@ -8828,10 +8828,10 @@
         <v/>
       </c>
       <c r="K154" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L154" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M154" s="8">
         <f>K154&amp;"-"&amp;L154</f>
@@ -8883,10 +8883,10 @@
         <v/>
       </c>
       <c r="K155" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L155" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M155" s="8">
         <f>K155&amp;"-"&amp;L155</f>
@@ -8938,10 +8938,10 @@
         <v/>
       </c>
       <c r="K156" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L156" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M156" s="8">
         <f>K156&amp;"-"&amp;L156</f>
@@ -8993,10 +8993,10 @@
         <v/>
       </c>
       <c r="K157" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L157" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M157" s="8">
         <f>K157&amp;"-"&amp;L157</f>
@@ -9048,10 +9048,10 @@
         <v/>
       </c>
       <c r="K158" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L158" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M158" s="8">
         <f>K158&amp;"-"&amp;L158</f>
@@ -9103,10 +9103,10 @@
         <v/>
       </c>
       <c r="K159" s="8" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L159" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M159" s="8">
         <f>K159&amp;"-"&amp;L159</f>
@@ -9158,10 +9158,10 @@
         <v/>
       </c>
       <c r="K160" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L160" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M160" s="8">
         <f>K160&amp;"-"&amp;L160</f>
@@ -9213,10 +9213,10 @@
         <v/>
       </c>
       <c r="K161" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L161" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M161" s="8">
         <f>K161&amp;"-"&amp;L161</f>
@@ -9268,10 +9268,10 @@
         <v/>
       </c>
       <c r="K162" s="8" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L162" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M162" s="8">
         <f>K162&amp;"-"&amp;L162</f>
@@ -9323,10 +9323,10 @@
         <v/>
       </c>
       <c r="K163" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L163" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M163" s="8">
         <f>K163&amp;"-"&amp;L163</f>
@@ -9378,10 +9378,10 @@
         <v/>
       </c>
       <c r="K164" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L164" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M164" s="8">
         <f>K164&amp;"-"&amp;L164</f>
@@ -9433,10 +9433,10 @@
         <v/>
       </c>
       <c r="K165" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L165" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M165" s="8">
         <f>K165&amp;"-"&amp;L165</f>
@@ -9488,10 +9488,10 @@
         <v/>
       </c>
       <c r="K166" s="8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L166" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M166" s="8">
         <f>K166&amp;"-"&amp;L166</f>
@@ -9543,10 +9543,10 @@
         <v/>
       </c>
       <c r="K167" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L167" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M167" s="8">
         <f>K167&amp;"-"&amp;L167</f>
@@ -9598,10 +9598,10 @@
         <v/>
       </c>
       <c r="K168" s="8" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L168" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M168" s="8">
         <f>K168&amp;"-"&amp;L168</f>
@@ -9653,10 +9653,10 @@
         <v/>
       </c>
       <c r="K169" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L169" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M169" s="8">
         <f>K169&amp;"-"&amp;L169</f>
@@ -9708,10 +9708,10 @@
         <v/>
       </c>
       <c r="K170" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L170" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M170" s="8">
         <f>K170&amp;"-"&amp;L170</f>
@@ -9763,10 +9763,10 @@
         <v/>
       </c>
       <c r="K171" s="8" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="L171" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M171" s="8">
         <f>K171&amp;"-"&amp;L171</f>
@@ -9818,10 +9818,10 @@
         <v/>
       </c>
       <c r="K172" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L172" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M172" s="8">
         <f>K172&amp;"-"&amp;L172</f>
@@ -9873,10 +9873,10 @@
         <v/>
       </c>
       <c r="K173" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L173" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M173" s="8">
         <f>K173&amp;"-"&amp;L173</f>
@@ -9928,10 +9928,10 @@
         <v/>
       </c>
       <c r="K174" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L174" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M174" s="8">
         <f>K174&amp;"-"&amp;L174</f>
@@ -10006,7 +10006,7 @@
     <row r="178">
       <c r="A178" s="11" t="inlineStr">
         <is>
-          <t>Teams with no games vs top 40</t>
+          <t>Teams with no November games vs top 40</t>
         </is>
       </c>
       <c r="B178" s="11" t="n"/>

</xml_diff>